<commit_message>
Atualiza preços de 2026-08-24
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,9 +469,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>403 Client Error: Forbidden for url: https://api.mercadolibre.com/sites/MLB/search?q=geladeira+brastemp+frost+free+375l&amp;limit=3</t>
@@ -494,9 +491,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>403 Client Error: Forbidden for url: https://www.casasbahia.com.br/api/catalog_system/pub/products/search/geladeira%20brastemp%20frost%20free%20375l</t>
@@ -519,9 +513,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>503 Server Error: Service Unavailable for url: https://www.fastshop.com.br/api/catalog_system/pub/products/search/geladeira%20brastemp%20frost%20free%20375l</t>
@@ -544,9 +535,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>nenhum resultado</t>
@@ -569,9 +557,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>nenhum resultado (pode ser bloqueio anti-robô)</t>
@@ -594,9 +579,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>403 Client Error: Forbidden for url: https://api.mercadolibre.com/sites/MLB/search?q=micro-ondas+electrolux+20l&amp;limit=3</t>
@@ -619,9 +601,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>403 Client Error: Forbidden for url: https://www.casasbahia.com.br/api/catalog_system/pub/products/search/micro-ondas%20electrolux%2020l</t>
@@ -644,9 +623,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>503 Server Error: Service Unavailable for url: https://www.fastshop.com.br/api/catalog_system/pub/products/search/micro-ondas%20electrolux%2020l</t>
@@ -669,9 +645,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>nenhum resultado</t>
@@ -694,9 +667,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>nenhum resultado (pode ser bloqueio anti-robô)</t>
@@ -719,9 +689,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
           <t>403 Client Error: Forbidden for url: https://api.mercadolibre.com/sites/MLB/search?q=fog%C3%A3o+4+bocas+consul&amp;limit=3</t>
@@ -744,9 +711,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>403 Client Error: Forbidden for url: https://www.casasbahia.com.br/api/catalog_system/pub/products/search/fog%C3%A3o%204%20bocas%20consul</t>
@@ -769,9 +733,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>503 Server Error: Service Unavailable for url: https://www.fastshop.com.br/api/catalog_system/pub/products/search/fog%C3%A3o%204%20bocas%20consul</t>
@@ -794,9 +755,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>nenhum resultado</t>
@@ -819,14 +777,518 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
           <t>nenhum resultado (pode ser bloqueio anti-robô)</t>
         </is>
       </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='api.scraperapi.com', port=443): Read timed out. (read timeout=30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Expecting value: line 1 column 1 (char 0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='api.scraperapi.com', port=443): Read timed out. (read timeout=30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>500 Server Error: Internal Server Error for url: https://api.scraperapi.com/?api_key=a35cd3114de750dd44e4af7aeb821045&amp;url=https%3A%2F%2Fwww.magazineluiza.com.br%2Fbusca%2Fgeladeira%2Bbrastemp%2Bfrost%2Bfree%2B375l%2F&amp;render=true</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWSXQGL/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Refrigerador-Brastemp-Duplex-Litros/dp/B07ND4BB3C/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='api.scraperapi.com', port=443): Read timed out. (read timeout=30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Expecting value: line 1 column 1 (char 0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='api.scraperapi.com', port=443): Read timed out. (read timeout=30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>500 Server Error: Internal Server Error for url: https://api.scraperapi.com/?api_key=a35cd3114de750dd44e4af7aeb821045&amp;url=https%3A%2F%2Fwww.magazineluiza.com.br%2Fbusca%2Fmicro-ondas%2Belectrolux%2B20l%2F&amp;render=true</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-MTO30-Fun%C3%A7%C3%A3o-Tira/dp/B083ZFFC5Q/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_2_so_MICROWAVE_OVEN</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='api.scraperapi.com', port=443): Read timed out. (read timeout=30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Expecting value: line 1 column 1 (char 0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='api.scraperapi.com', port=443): Read timed out. (read timeout=30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='api.scraperapi.com', port=443): Read timed out. (read timeout=60)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualiza preços de 2026-08-27
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G121"/>
+  <dimension ref="A1:G142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2728,9 +2728,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr"/>
-      <c r="E101" t="inlineStr"/>
-      <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
           <t>403 do proxy: 'Your current plan does not allow you to use our premium proxies. Please upgrade your plan to gain access to our Premium and Ultra Premium pools. More information can be found in our documentation https://docs.scraperapi.com/control-and-optimization/premium-residential-mobile-proxy-pools.'</t>
@@ -2753,9 +2750,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D102" t="inlineStr"/>
-      <c r="E102" t="inlineStr"/>
-      <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
           <t>403 do proxy: 'Your current plan does not allow you to use our premium proxies. Please upgrade your plan to gain access to our Premium and Ultra Premium pools. More information can be found in our documentation https://docs.scraperapi.com/control-and-optimization/premium-residential-mobile-proxy-pools.'</t>
@@ -2778,9 +2772,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D103" t="inlineStr"/>
-      <c r="E103" t="inlineStr"/>
-      <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
           <t>403 do proxy: 'Your current plan does not allow you to use our premium proxies. Please upgrade your plan to gain access to our Premium and Ultra Premium pools. More information can be found in our documentation https://docs.scraperapi.com/control-and-optimization/premium-residential-mobile-proxy-pools.'</t>
@@ -2803,9 +2794,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D104" t="inlineStr"/>
-      <c r="E104" t="inlineStr"/>
-      <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
           <t>403 do proxy: 'Your current plan does not allow you to use our premium proxies. Please upgrade your plan to gain access to our Premium and Ultra Premium pools. More information can be found in our documentation https://docs.scraperapi.com/control-and-optimization/premium-residential-mobile-proxy-pools.'</t>
@@ -2836,7 +2824,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -2862,7 +2849,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWSXQGL/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -2888,7 +2874,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWVJ8LR/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -2906,9 +2891,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr"/>
-      <c r="E108" t="inlineStr"/>
-      <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
           <t>403 do proxy: 'Your current plan does not allow you to use our premium proxies. Please upgrade your plan to gain access to our Premium and Ultra Premium pools. More information can be found in our documentation https://docs.scraperapi.com/control-and-optimization/premium-residential-mobile-proxy-pools.'</t>
@@ -2931,9 +2913,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D109" t="inlineStr"/>
-      <c r="E109" t="inlineStr"/>
-      <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
           <t>403 do proxy: 'Your current plan does not allow you to use our premium proxies. Please upgrade your plan to gain access to our Premium and Ultra Premium pools. More information can be found in our documentation https://docs.scraperapi.com/control-and-optimization/premium-residential-mobile-proxy-pools.'</t>
@@ -2956,9 +2935,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D110" t="inlineStr"/>
-      <c r="E110" t="inlineStr"/>
-      <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
           <t>403 do proxy: 'Your current plan does not allow you to use our premium proxies. Please upgrade your plan to gain access to our Premium and Ultra Premium pools. More information can be found in our documentation https://docs.scraperapi.com/control-and-optimization/premium-residential-mobile-proxy-pools.'</t>
@@ -2981,9 +2957,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D111" t="inlineStr"/>
-      <c r="E111" t="inlineStr"/>
-      <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
           <t>403 do proxy: 'Your current plan does not allow you to use our premium proxies. Please upgrade your plan to gain access to our Premium and Ultra Premium pools. More information can be found in our documentation https://docs.scraperapi.com/control-and-optimization/premium-residential-mobile-proxy-pools.'</t>
@@ -3014,7 +2987,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-MTO30-Fun%C3%A7%C3%A3o-Tira/dp/B083ZFFC5Q/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -3040,7 +3012,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -3066,7 +3037,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_2_so_MICROWAVE_OVEN</t>
         </is>
       </c>
-      <c r="G114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -3084,9 +3054,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D115" t="inlineStr"/>
-      <c r="E115" t="inlineStr"/>
-      <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr">
         <is>
           <t>403 do proxy: 'Your current plan does not allow you to use our premium proxies. Please upgrade your plan to gain access to our Premium and Ultra Premium pools. More information can be found in our documentation https://docs.scraperapi.com/control-and-optimization/premium-residential-mobile-proxy-pools.'</t>
@@ -3109,9 +3076,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D116" t="inlineStr"/>
-      <c r="E116" t="inlineStr"/>
-      <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
         <is>
           <t>403 do proxy: 'Your current plan does not allow you to use our premium proxies. Please upgrade your plan to gain access to our Premium and Ultra Premium pools. More information can be found in our documentation https://docs.scraperapi.com/control-and-optimization/premium-residential-mobile-proxy-pools.'</t>
@@ -3134,9 +3098,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D117" t="inlineStr"/>
-      <c r="E117" t="inlineStr"/>
-      <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
           <t>403 do proxy: 'Your current plan does not allow you to use our premium proxies. Please upgrade your plan to gain access to our Premium and Ultra Premium pools. More information can be found in our documentation https://docs.scraperapi.com/control-and-optimization/premium-residential-mobile-proxy-pools.'</t>
@@ -3159,9 +3120,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D118" t="inlineStr"/>
-      <c r="E118" t="inlineStr"/>
-      <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
         <is>
           <t>403 do proxy: 'Your current plan does not allow you to use our premium proxies. Please upgrade your plan to gain access to our Premium and Ultra Premium pools. More information can be found in our documentation https://docs.scraperapi.com/control-and-optimization/premium-residential-mobile-proxy-pools.'</t>
@@ -3192,7 +3150,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -3218,7 +3175,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -3244,7 +3200,540 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr"/>
+      <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr"/>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr"/>
+      <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr"/>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr"/>
+      <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr"/>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr"/>
+      <c r="E125" t="inlineStr"/>
+      <c r="F125" t="inlineStr"/>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E126" t="n">
+        <v>2599</v>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E127" t="n">
+        <v>3051.58</v>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWSXQGL/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>2849.99</v>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWVJ8LR/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr"/>
+      <c r="E129" t="inlineStr"/>
+      <c r="F129" t="inlineStr"/>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr"/>
+      <c r="E130" t="inlineStr"/>
+      <c r="F130" t="inlineStr"/>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr"/>
+      <c r="E131" t="inlineStr"/>
+      <c r="F131" t="inlineStr"/>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr"/>
+      <c r="E132" t="inlineStr"/>
+      <c r="F132" t="inlineStr"/>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>463</v>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_5</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E134" t="n">
+        <v>463</v>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_5_so_MICROWAVE_OVEN</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E135" t="n">
+        <v>513.13</v>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P3T3VM/ref=sr_1_6</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr"/>
+      <c r="E136" t="inlineStr"/>
+      <c r="F136" t="inlineStr"/>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr"/>
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr"/>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr"/>
+      <c r="E138" t="inlineStr"/>
+      <c r="F138" t="inlineStr"/>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr"/>
+      <c r="E139" t="inlineStr"/>
+      <c r="F139" t="inlineStr"/>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E140" t="n">
+        <v>1503.06</v>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E141" t="n">
+        <v>1448</v>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E142" t="n">
+        <v>1064</v>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualiza preços de 2026-08-28
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G142"/>
+  <dimension ref="A1:G163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3217,9 +3217,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D122" t="inlineStr"/>
-      <c r="E122" t="inlineStr"/>
-      <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -3242,9 +3239,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D123" t="inlineStr"/>
-      <c r="E123" t="inlineStr"/>
-      <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -3267,9 +3261,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D124" t="inlineStr"/>
-      <c r="E124" t="inlineStr"/>
-      <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -3292,9 +3283,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D125" t="inlineStr"/>
-      <c r="E125" t="inlineStr"/>
-      <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -3325,7 +3313,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -3351,7 +3338,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWSXQGL/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -3377,7 +3363,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWVJ8LR/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -3395,9 +3380,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D129" t="inlineStr"/>
-      <c r="E129" t="inlineStr"/>
-      <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -3420,9 +3402,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D130" t="inlineStr"/>
-      <c r="E130" t="inlineStr"/>
-      <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -3445,9 +3424,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D131" t="inlineStr"/>
-      <c r="E131" t="inlineStr"/>
-      <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -3470,9 +3446,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D132" t="inlineStr"/>
-      <c r="E132" t="inlineStr"/>
-      <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -3503,7 +3476,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_5</t>
         </is>
       </c>
-      <c r="G133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -3529,7 +3501,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_5_so_MICROWAVE_OVEN</t>
         </is>
       </c>
-      <c r="G134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -3555,7 +3526,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P3T3VM/ref=sr_1_6</t>
         </is>
       </c>
-      <c r="G135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -3573,9 +3543,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D136" t="inlineStr"/>
-      <c r="E136" t="inlineStr"/>
-      <c r="F136" t="inlineStr"/>
       <c r="G136" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -3598,9 +3565,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D137" t="inlineStr"/>
-      <c r="E137" t="inlineStr"/>
-      <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -3623,9 +3587,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D138" t="inlineStr"/>
-      <c r="E138" t="inlineStr"/>
-      <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -3648,9 +3609,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D139" t="inlineStr"/>
-      <c r="E139" t="inlineStr"/>
-      <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -3681,7 +3639,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -3707,7 +3664,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -3733,7 +3689,540 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr"/>
+      <c r="E143" t="inlineStr"/>
+      <c r="F143" t="inlineStr"/>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr"/>
+      <c r="E144" t="inlineStr"/>
+      <c r="F144" t="inlineStr"/>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr"/>
+      <c r="E145" t="inlineStr"/>
+      <c r="F145" t="inlineStr"/>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr"/>
+      <c r="E146" t="inlineStr"/>
+      <c r="F146" t="inlineStr"/>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E147" t="n">
+        <v>2658.98</v>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E148" t="n">
+        <v>3299</v>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWSXQGL/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E149" t="n">
+        <v>3332.22</v>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWVJ8LR/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr"/>
+      <c r="E150" t="inlineStr"/>
+      <c r="F150" t="inlineStr"/>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr"/>
+      <c r="E151" t="inlineStr"/>
+      <c r="F151" t="inlineStr"/>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr"/>
+      <c r="E152" t="inlineStr"/>
+      <c r="F152" t="inlineStr"/>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr"/>
+      <c r="E153" t="inlineStr"/>
+      <c r="F153" t="inlineStr"/>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E154" t="n">
+        <v>499</v>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E155" t="n">
+        <v>499</v>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_1_so_MICROWAVE_OVEN</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E156" t="n">
+        <v>524.02</v>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P3T3VM/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr"/>
+      <c r="E157" t="inlineStr"/>
+      <c r="F157" t="inlineStr"/>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr"/>
+      <c r="E158" t="inlineStr"/>
+      <c r="F158" t="inlineStr"/>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr"/>
+      <c r="E159" t="inlineStr"/>
+      <c r="F159" t="inlineStr"/>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr"/>
+      <c r="E160" t="inlineStr"/>
+      <c r="F160" t="inlineStr"/>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E161" t="n">
+        <v>1278.9</v>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E162" t="n">
+        <v>1448</v>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E163" t="n">
+        <v>1064</v>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualiza preços de 2026-08-29
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G163"/>
+  <dimension ref="A1:G184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3706,9 +3706,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D143" t="inlineStr"/>
-      <c r="E143" t="inlineStr"/>
-      <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -3731,9 +3728,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D144" t="inlineStr"/>
-      <c r="E144" t="inlineStr"/>
-      <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -3756,9 +3750,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D145" t="inlineStr"/>
-      <c r="E145" t="inlineStr"/>
-      <c r="F145" t="inlineStr"/>
       <c r="G145" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -3781,9 +3772,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D146" t="inlineStr"/>
-      <c r="E146" t="inlineStr"/>
-      <c r="F146" t="inlineStr"/>
       <c r="G146" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -3814,7 +3802,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -3840,7 +3827,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWSXQGL/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -3866,7 +3852,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWVJ8LR/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -3884,9 +3869,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D150" t="inlineStr"/>
-      <c r="E150" t="inlineStr"/>
-      <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -3909,9 +3891,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D151" t="inlineStr"/>
-      <c r="E151" t="inlineStr"/>
-      <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -3934,9 +3913,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D152" t="inlineStr"/>
-      <c r="E152" t="inlineStr"/>
-      <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -3959,9 +3935,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D153" t="inlineStr"/>
-      <c r="E153" t="inlineStr"/>
-      <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -3992,7 +3965,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -4018,7 +3990,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_1_so_MICROWAVE_OVEN</t>
         </is>
       </c>
-      <c r="G155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -4044,7 +4015,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P3T3VM/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -4062,9 +4032,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D157" t="inlineStr"/>
-      <c r="E157" t="inlineStr"/>
-      <c r="F157" t="inlineStr"/>
       <c r="G157" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -4087,9 +4054,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D158" t="inlineStr"/>
-      <c r="E158" t="inlineStr"/>
-      <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -4112,9 +4076,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D159" t="inlineStr"/>
-      <c r="E159" t="inlineStr"/>
-      <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -4137,9 +4098,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D160" t="inlineStr"/>
-      <c r="E160" t="inlineStr"/>
-      <c r="F160" t="inlineStr"/>
       <c r="G160" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -4170,7 +4128,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -4196,7 +4153,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -4222,7 +4178,540 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr"/>
+      <c r="E164" t="inlineStr"/>
+      <c r="F164" t="inlineStr"/>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr"/>
+      <c r="E165" t="inlineStr"/>
+      <c r="F165" t="inlineStr"/>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr"/>
+      <c r="E166" t="inlineStr"/>
+      <c r="F166" t="inlineStr"/>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr"/>
+      <c r="E167" t="inlineStr"/>
+      <c r="F167" t="inlineStr"/>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E168" t="n">
+        <v>2658.98</v>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E169" t="n">
+        <v>3299</v>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWSXQGL/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E170" t="n">
+        <v>2849.99</v>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWVJ8LR/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr"/>
+      <c r="E171" t="inlineStr"/>
+      <c r="F171" t="inlineStr"/>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr"/>
+      <c r="E172" t="inlineStr"/>
+      <c r="F172" t="inlineStr"/>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr"/>
+      <c r="E173" t="inlineStr"/>
+      <c r="F173" t="inlineStr"/>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr"/>
+      <c r="E174" t="inlineStr"/>
+      <c r="F174" t="inlineStr"/>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E175" t="n">
+        <v>499</v>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E176" t="n">
+        <v>499</v>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_1_so_MICROWAVE_OVEN</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E177" t="n">
+        <v>513.13</v>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P3T3VM/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr"/>
+      <c r="E178" t="inlineStr"/>
+      <c r="F178" t="inlineStr"/>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr"/>
+      <c r="E179" t="inlineStr"/>
+      <c r="F179" t="inlineStr"/>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr"/>
+      <c r="E180" t="inlineStr"/>
+      <c r="F180" t="inlineStr"/>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr"/>
+      <c r="E181" t="inlineStr"/>
+      <c r="F181" t="inlineStr"/>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E182" t="n">
+        <v>1278.9</v>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_5</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E183" t="n">
+        <v>1278.9</v>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_6</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr"/>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E184" t="n">
+        <v>1064</v>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_7</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualiza preços de 2026-08-30
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G184"/>
+  <dimension ref="A1:G205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4195,9 +4195,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D164" t="inlineStr"/>
-      <c r="E164" t="inlineStr"/>
-      <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -4220,9 +4217,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D165" t="inlineStr"/>
-      <c r="E165" t="inlineStr"/>
-      <c r="F165" t="inlineStr"/>
       <c r="G165" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -4245,9 +4239,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D166" t="inlineStr"/>
-      <c r="E166" t="inlineStr"/>
-      <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -4270,9 +4261,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D167" t="inlineStr"/>
-      <c r="E167" t="inlineStr"/>
-      <c r="F167" t="inlineStr"/>
       <c r="G167" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -4303,7 +4291,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -4329,7 +4316,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWSXQGL/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -4355,7 +4341,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWVJ8LR/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -4373,9 +4358,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D171" t="inlineStr"/>
-      <c r="E171" t="inlineStr"/>
-      <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -4398,9 +4380,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D172" t="inlineStr"/>
-      <c r="E172" t="inlineStr"/>
-      <c r="F172" t="inlineStr"/>
       <c r="G172" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -4423,9 +4402,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D173" t="inlineStr"/>
-      <c r="E173" t="inlineStr"/>
-      <c r="F173" t="inlineStr"/>
       <c r="G173" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -4448,9 +4424,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D174" t="inlineStr"/>
-      <c r="E174" t="inlineStr"/>
-      <c r="F174" t="inlineStr"/>
       <c r="G174" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -4481,7 +4454,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -4507,7 +4479,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_1_so_MICROWAVE_OVEN</t>
         </is>
       </c>
-      <c r="G176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -4533,7 +4504,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P3T3VM/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -4551,9 +4521,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D178" t="inlineStr"/>
-      <c r="E178" t="inlineStr"/>
-      <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -4576,9 +4543,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D179" t="inlineStr"/>
-      <c r="E179" t="inlineStr"/>
-      <c r="F179" t="inlineStr"/>
       <c r="G179" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -4601,9 +4565,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D180" t="inlineStr"/>
-      <c r="E180" t="inlineStr"/>
-      <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -4626,9 +4587,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D181" t="inlineStr"/>
-      <c r="E181" t="inlineStr"/>
-      <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -4659,7 +4617,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_5</t>
         </is>
       </c>
-      <c r="G182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -4685,7 +4642,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_6</t>
         </is>
       </c>
-      <c r="G183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -4711,7 +4667,540 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_7</t>
         </is>
       </c>
-      <c r="G184" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr"/>
+      <c r="E185" t="inlineStr"/>
+      <c r="F185" t="inlineStr"/>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr"/>
+      <c r="E186" t="inlineStr"/>
+      <c r="F186" t="inlineStr"/>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr"/>
+      <c r="E187" t="inlineStr"/>
+      <c r="F187" t="inlineStr"/>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr"/>
+      <c r="E188" t="inlineStr"/>
+      <c r="F188" t="inlineStr"/>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E189" t="n">
+        <v>2599</v>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_5</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr"/>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E190" t="n">
+        <v>3040.21</v>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWSXQGL/ref=sr_1_6</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr"/>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E191" t="n">
+        <v>2849.99</v>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWVJ8LR/ref=sr_1_7</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr"/>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr"/>
+      <c r="E192" t="inlineStr"/>
+      <c r="F192" t="inlineStr"/>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr"/>
+      <c r="E193" t="inlineStr"/>
+      <c r="F193" t="inlineStr"/>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr"/>
+      <c r="E194" t="inlineStr"/>
+      <c r="F194" t="inlineStr"/>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr"/>
+      <c r="E195" t="inlineStr"/>
+      <c r="F195" t="inlineStr"/>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E196" t="n">
+        <v>499</v>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E197" t="n">
+        <v>499</v>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_1_so_MICROWAVE_OVEN</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr"/>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E198" t="n">
+        <v>513.13</v>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P3T3VM/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr"/>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr"/>
+      <c r="E199" t="inlineStr"/>
+      <c r="F199" t="inlineStr"/>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr"/>
+      <c r="E200" t="inlineStr"/>
+      <c r="F200" t="inlineStr"/>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr"/>
+      <c r="E201" t="inlineStr"/>
+      <c r="F201" t="inlineStr"/>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr"/>
+      <c r="E202" t="inlineStr"/>
+      <c r="F202" t="inlineStr"/>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E203" t="n">
+        <v>1448</v>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E204" t="n">
+        <v>1064</v>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr"/>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E205" t="n">
+        <v>1245.5</v>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualiza preços de 2026-08-31
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G205"/>
+  <dimension ref="A1:G226"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4684,9 +4684,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D185" t="inlineStr"/>
-      <c r="E185" t="inlineStr"/>
-      <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -4709,9 +4706,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D186" t="inlineStr"/>
-      <c r="E186" t="inlineStr"/>
-      <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -4734,9 +4728,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D187" t="inlineStr"/>
-      <c r="E187" t="inlineStr"/>
-      <c r="F187" t="inlineStr"/>
       <c r="G187" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -4759,9 +4750,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D188" t="inlineStr"/>
-      <c r="E188" t="inlineStr"/>
-      <c r="F188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -4792,7 +4780,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_5</t>
         </is>
       </c>
-      <c r="G189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -4818,7 +4805,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWSXQGL/ref=sr_1_6</t>
         </is>
       </c>
-      <c r="G190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -4844,7 +4830,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWVJ8LR/ref=sr_1_7</t>
         </is>
       </c>
-      <c r="G191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -4862,9 +4847,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D192" t="inlineStr"/>
-      <c r="E192" t="inlineStr"/>
-      <c r="F192" t="inlineStr"/>
       <c r="G192" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -4887,9 +4869,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D193" t="inlineStr"/>
-      <c r="E193" t="inlineStr"/>
-      <c r="F193" t="inlineStr"/>
       <c r="G193" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -4912,9 +4891,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D194" t="inlineStr"/>
-      <c r="E194" t="inlineStr"/>
-      <c r="F194" t="inlineStr"/>
       <c r="G194" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -4937,9 +4913,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D195" t="inlineStr"/>
-      <c r="E195" t="inlineStr"/>
-      <c r="F195" t="inlineStr"/>
       <c r="G195" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -4970,7 +4943,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -4996,7 +4968,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_1_so_MICROWAVE_OVEN</t>
         </is>
       </c>
-      <c r="G197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -5022,7 +4993,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P3T3VM/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -5040,9 +5010,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D199" t="inlineStr"/>
-      <c r="E199" t="inlineStr"/>
-      <c r="F199" t="inlineStr"/>
       <c r="G199" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -5065,9 +5032,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D200" t="inlineStr"/>
-      <c r="E200" t="inlineStr"/>
-      <c r="F200" t="inlineStr"/>
       <c r="G200" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -5090,9 +5054,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D201" t="inlineStr"/>
-      <c r="E201" t="inlineStr"/>
-      <c r="F201" t="inlineStr"/>
       <c r="G201" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -5115,9 +5076,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D202" t="inlineStr"/>
-      <c r="E202" t="inlineStr"/>
-      <c r="F202" t="inlineStr"/>
       <c r="G202" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -5148,7 +5106,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -5174,7 +5131,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -5200,7 +5156,540 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G205" t="inlineStr"/>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr"/>
+      <c r="E206" t="inlineStr"/>
+      <c r="F206" t="inlineStr"/>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr"/>
+      <c r="E207" t="inlineStr"/>
+      <c r="F207" t="inlineStr"/>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr"/>
+      <c r="E208" t="inlineStr"/>
+      <c r="F208" t="inlineStr"/>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr"/>
+      <c r="E209" t="inlineStr"/>
+      <c r="F209" t="inlineStr"/>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E210" t="n">
+        <v>2658.98</v>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_1</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E211" t="n">
+        <v>3299</v>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWSXQGL/ref=sr_1_2</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr"/>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E212" t="n">
+        <v>3332.22</v>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWVJ8LR/ref=sr_1_3</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr"/>
+      <c r="E213" t="inlineStr"/>
+      <c r="F213" t="inlineStr"/>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr"/>
+      <c r="E214" t="inlineStr"/>
+      <c r="F214" t="inlineStr"/>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr"/>
+      <c r="E215" t="inlineStr"/>
+      <c r="F215" t="inlineStr"/>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr"/>
+      <c r="E216" t="inlineStr"/>
+      <c r="F216" t="inlineStr"/>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E217" t="n">
+        <v>499</v>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_4</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr"/>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E218" t="n">
+        <v>499</v>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_4_so_MICROWAVE_OVEN</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr"/>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E219" t="n">
+        <v>513.13</v>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P3T3VM/ref=sr_1_5</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr"/>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr"/>
+      <c r="E220" t="inlineStr"/>
+      <c r="F220" t="inlineStr"/>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr"/>
+      <c r="E221" t="inlineStr"/>
+      <c r="F221" t="inlineStr"/>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr"/>
+      <c r="E222" t="inlineStr"/>
+      <c r="F222" t="inlineStr"/>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr"/>
+      <c r="E223" t="inlineStr"/>
+      <c r="F223" t="inlineStr"/>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E224" t="n">
+        <v>1448</v>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_5</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr"/>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E225" t="n">
+        <v>1064</v>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_6</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr"/>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="E226" t="n">
+        <v>1329.3</v>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_7</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-01
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G226"/>
+  <dimension ref="A1:G241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5173,9 +5173,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D206" t="inlineStr"/>
-      <c r="E206" t="inlineStr"/>
-      <c r="F206" t="inlineStr"/>
       <c r="G206" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -5198,9 +5195,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D207" t="inlineStr"/>
-      <c r="E207" t="inlineStr"/>
-      <c r="F207" t="inlineStr"/>
       <c r="G207" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -5223,9 +5217,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D208" t="inlineStr"/>
-      <c r="E208" t="inlineStr"/>
-      <c r="F208" t="inlineStr"/>
       <c r="G208" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -5248,9 +5239,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D209" t="inlineStr"/>
-      <c r="E209" t="inlineStr"/>
-      <c r="F209" t="inlineStr"/>
       <c r="G209" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -5281,7 +5269,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Duplex-litros-Branca/dp/B07FXZ8TR6/ref=sr_1_1</t>
         </is>
       </c>
-      <c r="G210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -5307,7 +5294,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWSXQGL/ref=sr_1_2</t>
         </is>
       </c>
-      <c r="G211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -5333,7 +5319,6 @@
           <t>https://www.amazon.com.br/Geladeira-Brastemp-Frost-Duplex-litros/dp/B07GWVJ8LR/ref=sr_1_3</t>
         </is>
       </c>
-      <c r="G212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -5351,9 +5336,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D213" t="inlineStr"/>
-      <c r="E213" t="inlineStr"/>
-      <c r="F213" t="inlineStr"/>
       <c r="G213" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -5376,9 +5358,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D214" t="inlineStr"/>
-      <c r="E214" t="inlineStr"/>
-      <c r="F214" t="inlineStr"/>
       <c r="G214" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -5401,9 +5380,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D215" t="inlineStr"/>
-      <c r="E215" t="inlineStr"/>
-      <c r="F215" t="inlineStr"/>
       <c r="G215" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -5426,9 +5402,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D216" t="inlineStr"/>
-      <c r="E216" t="inlineStr"/>
-      <c r="F216" t="inlineStr"/>
       <c r="G216" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -5459,7 +5432,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_4</t>
         </is>
       </c>
-      <c r="G217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -5485,7 +5457,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Electrolux-Tira-Odor-MT30S/dp/B079Y3MLSP/ref=sr_1_4_so_MICROWAVE_OVEN</t>
         </is>
       </c>
-      <c r="G218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -5511,7 +5482,6 @@
           <t>https://www.amazon.com.br/Micro-ondas-Bancada-Electrolux-Efficient-ME23S/dp/B0B8P3T3VM/ref=sr_1_5</t>
         </is>
       </c>
-      <c r="G219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -5529,9 +5499,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D220" t="inlineStr"/>
-      <c r="E220" t="inlineStr"/>
-      <c r="F220" t="inlineStr"/>
       <c r="G220" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -5554,9 +5521,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D221" t="inlineStr"/>
-      <c r="E221" t="inlineStr"/>
-      <c r="F221" t="inlineStr"/>
       <c r="G221" t="inlineStr">
         <is>
           <t>resposta inválida do proxy (corpo vazio ou não-JSON)</t>
@@ -5579,9 +5543,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D222" t="inlineStr"/>
-      <c r="E222" t="inlineStr"/>
-      <c r="F222" t="inlineStr"/>
       <c r="G222" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -5604,9 +5565,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D223" t="inlineStr"/>
-      <c r="E223" t="inlineStr"/>
-      <c r="F223" t="inlineStr"/>
       <c r="G223" t="inlineStr">
         <is>
           <t>500 do proxy: 'Request failed. You will not be charged for this request. Please make sure your url is correct and try again. Protected domains may require adding premium=true OR ultra_premium=true parameter to your request.'</t>
@@ -5637,7 +5595,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Bocas-Consul-Vidro-Bivolt/dp/B076BC7769/ref=sr_1_5</t>
         </is>
       </c>
-      <c r="G224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -5663,7 +5620,6 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-04-Bocas-FS-CF04NABUNA/dp/B07JPZN51P/ref=sr_1_6</t>
         </is>
       </c>
-      <c r="G225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -5689,7 +5645,381 @@
           <t>https://www.amazon.com.br/Fog%C3%A3o-Consul-Bocas-CFO4NARUNA-Bivolt/dp/B07HM9JL5K/ref=sr_1_7</t>
         </is>
       </c>
-      <c r="G226" t="inlineStr"/>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr"/>
+      <c r="E227" t="inlineStr"/>
+      <c r="F227" t="inlineStr"/>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr"/>
+      <c r="E228" t="inlineStr"/>
+      <c r="F228" t="inlineStr"/>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr"/>
+      <c r="E229" t="inlineStr"/>
+      <c r="F229" t="inlineStr"/>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr"/>
+      <c r="E230" t="inlineStr"/>
+      <c r="F230" t="inlineStr"/>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr"/>
+      <c r="E231" t="inlineStr"/>
+      <c r="F231" t="inlineStr"/>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr"/>
+      <c r="E232" t="inlineStr"/>
+      <c r="F232" t="inlineStr"/>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr"/>
+      <c r="E233" t="inlineStr"/>
+      <c r="F233" t="inlineStr"/>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr"/>
+      <c r="E234" t="inlineStr"/>
+      <c r="F234" t="inlineStr"/>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr"/>
+      <c r="E235" t="inlineStr"/>
+      <c r="F235" t="inlineStr"/>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr"/>
+      <c r="E236" t="inlineStr"/>
+      <c r="F236" t="inlineStr"/>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr"/>
+      <c r="E237" t="inlineStr"/>
+      <c r="F237" t="inlineStr"/>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr"/>
+      <c r="E238" t="inlineStr"/>
+      <c r="F238" t="inlineStr"/>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr"/>
+      <c r="E239" t="inlineStr"/>
+      <c r="F239" t="inlineStr"/>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr"/>
+      <c r="E240" t="inlineStr"/>
+      <c r="F240" t="inlineStr"/>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr"/>
+      <c r="E241" t="inlineStr"/>
+      <c r="F241" t="inlineStr"/>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-02
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G241"/>
+  <dimension ref="A1:G256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5662,9 +5662,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D227" t="inlineStr"/>
-      <c r="E227" t="inlineStr"/>
-      <c r="F227" t="inlineStr"/>
       <c r="G227" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -5687,9 +5684,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D228" t="inlineStr"/>
-      <c r="E228" t="inlineStr"/>
-      <c r="F228" t="inlineStr"/>
       <c r="G228" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -5712,9 +5706,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D229" t="inlineStr"/>
-      <c r="E229" t="inlineStr"/>
-      <c r="F229" t="inlineStr"/>
       <c r="G229" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -5737,9 +5728,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D230" t="inlineStr"/>
-      <c r="E230" t="inlineStr"/>
-      <c r="F230" t="inlineStr"/>
       <c r="G230" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -5762,9 +5750,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D231" t="inlineStr"/>
-      <c r="E231" t="inlineStr"/>
-      <c r="F231" t="inlineStr"/>
       <c r="G231" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -5787,9 +5772,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D232" t="inlineStr"/>
-      <c r="E232" t="inlineStr"/>
-      <c r="F232" t="inlineStr"/>
       <c r="G232" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -5812,9 +5794,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D233" t="inlineStr"/>
-      <c r="E233" t="inlineStr"/>
-      <c r="F233" t="inlineStr"/>
       <c r="G233" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -5837,9 +5816,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D234" t="inlineStr"/>
-      <c r="E234" t="inlineStr"/>
-      <c r="F234" t="inlineStr"/>
       <c r="G234" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -5862,9 +5838,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D235" t="inlineStr"/>
-      <c r="E235" t="inlineStr"/>
-      <c r="F235" t="inlineStr"/>
       <c r="G235" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -5887,9 +5860,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D236" t="inlineStr"/>
-      <c r="E236" t="inlineStr"/>
-      <c r="F236" t="inlineStr"/>
       <c r="G236" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -5912,9 +5882,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D237" t="inlineStr"/>
-      <c r="E237" t="inlineStr"/>
-      <c r="F237" t="inlineStr"/>
       <c r="G237" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -5937,9 +5904,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D238" t="inlineStr"/>
-      <c r="E238" t="inlineStr"/>
-      <c r="F238" t="inlineStr"/>
       <c r="G238" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -5962,9 +5926,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D239" t="inlineStr"/>
-      <c r="E239" t="inlineStr"/>
-      <c r="F239" t="inlineStr"/>
       <c r="G239" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -5987,9 +5948,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D240" t="inlineStr"/>
-      <c r="E240" t="inlineStr"/>
-      <c r="F240" t="inlineStr"/>
       <c r="G240" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6012,10 +5970,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D241" t="inlineStr"/>
-      <c r="E241" t="inlineStr"/>
-      <c r="F241" t="inlineStr"/>
       <c r="G241" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr"/>
+      <c r="E242" t="inlineStr"/>
+      <c r="F242" t="inlineStr"/>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr"/>
+      <c r="E243" t="inlineStr"/>
+      <c r="F243" t="inlineStr"/>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr"/>
+      <c r="E244" t="inlineStr"/>
+      <c r="F244" t="inlineStr"/>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr"/>
+      <c r="E245" t="inlineStr"/>
+      <c r="F245" t="inlineStr"/>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr"/>
+      <c r="E246" t="inlineStr"/>
+      <c r="F246" t="inlineStr"/>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr"/>
+      <c r="E247" t="inlineStr"/>
+      <c r="F247" t="inlineStr"/>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr"/>
+      <c r="E248" t="inlineStr"/>
+      <c r="F248" t="inlineStr"/>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr"/>
+      <c r="E249" t="inlineStr"/>
+      <c r="F249" t="inlineStr"/>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr"/>
+      <c r="E250" t="inlineStr"/>
+      <c r="F250" t="inlineStr"/>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr"/>
+      <c r="E251" t="inlineStr"/>
+      <c r="F251" t="inlineStr"/>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr"/>
+      <c r="E252" t="inlineStr"/>
+      <c r="F252" t="inlineStr"/>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr"/>
+      <c r="E253" t="inlineStr"/>
+      <c r="F253" t="inlineStr"/>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr"/>
+      <c r="E254" t="inlineStr"/>
+      <c r="F254" t="inlineStr"/>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr"/>
+      <c r="E255" t="inlineStr"/>
+      <c r="F255" t="inlineStr"/>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr"/>
+      <c r="E256" t="inlineStr"/>
+      <c r="F256" t="inlineStr"/>
+      <c r="G256" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-03
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G256"/>
+  <dimension ref="A1:G271"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5992,9 +5992,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D242" t="inlineStr"/>
-      <c r="E242" t="inlineStr"/>
-      <c r="F242" t="inlineStr"/>
       <c r="G242" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6017,9 +6014,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D243" t="inlineStr"/>
-      <c r="E243" t="inlineStr"/>
-      <c r="F243" t="inlineStr"/>
       <c r="G243" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6042,9 +6036,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D244" t="inlineStr"/>
-      <c r="E244" t="inlineStr"/>
-      <c r="F244" t="inlineStr"/>
       <c r="G244" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6067,9 +6058,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D245" t="inlineStr"/>
-      <c r="E245" t="inlineStr"/>
-      <c r="F245" t="inlineStr"/>
       <c r="G245" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6092,9 +6080,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D246" t="inlineStr"/>
-      <c r="E246" t="inlineStr"/>
-      <c r="F246" t="inlineStr"/>
       <c r="G246" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6117,9 +6102,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D247" t="inlineStr"/>
-      <c r="E247" t="inlineStr"/>
-      <c r="F247" t="inlineStr"/>
       <c r="G247" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6142,9 +6124,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D248" t="inlineStr"/>
-      <c r="E248" t="inlineStr"/>
-      <c r="F248" t="inlineStr"/>
       <c r="G248" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6167,9 +6146,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D249" t="inlineStr"/>
-      <c r="E249" t="inlineStr"/>
-      <c r="F249" t="inlineStr"/>
       <c r="G249" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6192,9 +6168,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D250" t="inlineStr"/>
-      <c r="E250" t="inlineStr"/>
-      <c r="F250" t="inlineStr"/>
       <c r="G250" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6217,9 +6190,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D251" t="inlineStr"/>
-      <c r="E251" t="inlineStr"/>
-      <c r="F251" t="inlineStr"/>
       <c r="G251" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6242,9 +6212,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D252" t="inlineStr"/>
-      <c r="E252" t="inlineStr"/>
-      <c r="F252" t="inlineStr"/>
       <c r="G252" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6267,9 +6234,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D253" t="inlineStr"/>
-      <c r="E253" t="inlineStr"/>
-      <c r="F253" t="inlineStr"/>
       <c r="G253" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6292,9 +6256,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D254" t="inlineStr"/>
-      <c r="E254" t="inlineStr"/>
-      <c r="F254" t="inlineStr"/>
       <c r="G254" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6317,9 +6278,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D255" t="inlineStr"/>
-      <c r="E255" t="inlineStr"/>
-      <c r="F255" t="inlineStr"/>
       <c r="G255" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6342,10 +6300,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D256" t="inlineStr"/>
-      <c r="E256" t="inlineStr"/>
-      <c r="F256" t="inlineStr"/>
       <c r="G256" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr"/>
+      <c r="E257" t="inlineStr"/>
+      <c r="F257" t="inlineStr"/>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr"/>
+      <c r="E258" t="inlineStr"/>
+      <c r="F258" t="inlineStr"/>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr"/>
+      <c r="E259" t="inlineStr"/>
+      <c r="F259" t="inlineStr"/>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr"/>
+      <c r="E260" t="inlineStr"/>
+      <c r="F260" t="inlineStr"/>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr"/>
+      <c r="E261" t="inlineStr"/>
+      <c r="F261" t="inlineStr"/>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr"/>
+      <c r="E262" t="inlineStr"/>
+      <c r="F262" t="inlineStr"/>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr"/>
+      <c r="E263" t="inlineStr"/>
+      <c r="F263" t="inlineStr"/>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr"/>
+      <c r="E264" t="inlineStr"/>
+      <c r="F264" t="inlineStr"/>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr"/>
+      <c r="E265" t="inlineStr"/>
+      <c r="F265" t="inlineStr"/>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr"/>
+      <c r="E266" t="inlineStr"/>
+      <c r="F266" t="inlineStr"/>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr"/>
+      <c r="E267" t="inlineStr"/>
+      <c r="F267" t="inlineStr"/>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr"/>
+      <c r="E268" t="inlineStr"/>
+      <c r="F268" t="inlineStr"/>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr"/>
+      <c r="E269" t="inlineStr"/>
+      <c r="F269" t="inlineStr"/>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr"/>
+      <c r="E270" t="inlineStr"/>
+      <c r="F270" t="inlineStr"/>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr"/>
+      <c r="E271" t="inlineStr"/>
+      <c r="F271" t="inlineStr"/>
+      <c r="G271" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-04
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G271"/>
+  <dimension ref="A1:G286"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6322,9 +6322,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D257" t="inlineStr"/>
-      <c r="E257" t="inlineStr"/>
-      <c r="F257" t="inlineStr"/>
       <c r="G257" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6347,9 +6344,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D258" t="inlineStr"/>
-      <c r="E258" t="inlineStr"/>
-      <c r="F258" t="inlineStr"/>
       <c r="G258" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6372,9 +6366,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D259" t="inlineStr"/>
-      <c r="E259" t="inlineStr"/>
-      <c r="F259" t="inlineStr"/>
       <c r="G259" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6397,9 +6388,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D260" t="inlineStr"/>
-      <c r="E260" t="inlineStr"/>
-      <c r="F260" t="inlineStr"/>
       <c r="G260" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6422,9 +6410,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D261" t="inlineStr"/>
-      <c r="E261" t="inlineStr"/>
-      <c r="F261" t="inlineStr"/>
       <c r="G261" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6447,9 +6432,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D262" t="inlineStr"/>
-      <c r="E262" t="inlineStr"/>
-      <c r="F262" t="inlineStr"/>
       <c r="G262" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6472,9 +6454,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D263" t="inlineStr"/>
-      <c r="E263" t="inlineStr"/>
-      <c r="F263" t="inlineStr"/>
       <c r="G263" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6497,9 +6476,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D264" t="inlineStr"/>
-      <c r="E264" t="inlineStr"/>
-      <c r="F264" t="inlineStr"/>
       <c r="G264" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6522,9 +6498,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D265" t="inlineStr"/>
-      <c r="E265" t="inlineStr"/>
-      <c r="F265" t="inlineStr"/>
       <c r="G265" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6547,9 +6520,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D266" t="inlineStr"/>
-      <c r="E266" t="inlineStr"/>
-      <c r="F266" t="inlineStr"/>
       <c r="G266" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6572,9 +6542,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D267" t="inlineStr"/>
-      <c r="E267" t="inlineStr"/>
-      <c r="F267" t="inlineStr"/>
       <c r="G267" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6597,9 +6564,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D268" t="inlineStr"/>
-      <c r="E268" t="inlineStr"/>
-      <c r="F268" t="inlineStr"/>
       <c r="G268" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6622,9 +6586,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D269" t="inlineStr"/>
-      <c r="E269" t="inlineStr"/>
-      <c r="F269" t="inlineStr"/>
       <c r="G269" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6647,9 +6608,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D270" t="inlineStr"/>
-      <c r="E270" t="inlineStr"/>
-      <c r="F270" t="inlineStr"/>
       <c r="G270" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6672,10 +6630,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D271" t="inlineStr"/>
-      <c r="E271" t="inlineStr"/>
-      <c r="F271" t="inlineStr"/>
       <c r="G271" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr"/>
+      <c r="E272" t="inlineStr"/>
+      <c r="F272" t="inlineStr"/>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr"/>
+      <c r="E273" t="inlineStr"/>
+      <c r="F273" t="inlineStr"/>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr"/>
+      <c r="E274" t="inlineStr"/>
+      <c r="F274" t="inlineStr"/>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr"/>
+      <c r="E275" t="inlineStr"/>
+      <c r="F275" t="inlineStr"/>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr"/>
+      <c r="E276" t="inlineStr"/>
+      <c r="F276" t="inlineStr"/>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr"/>
+      <c r="E277" t="inlineStr"/>
+      <c r="F277" t="inlineStr"/>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr"/>
+      <c r="E278" t="inlineStr"/>
+      <c r="F278" t="inlineStr"/>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr"/>
+      <c r="E279" t="inlineStr"/>
+      <c r="F279" t="inlineStr"/>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr"/>
+      <c r="E280" t="inlineStr"/>
+      <c r="F280" t="inlineStr"/>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr"/>
+      <c r="E281" t="inlineStr"/>
+      <c r="F281" t="inlineStr"/>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr"/>
+      <c r="E282" t="inlineStr"/>
+      <c r="F282" t="inlineStr"/>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr"/>
+      <c r="E283" t="inlineStr"/>
+      <c r="F283" t="inlineStr"/>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr"/>
+      <c r="E284" t="inlineStr"/>
+      <c r="F284" t="inlineStr"/>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr"/>
+      <c r="E285" t="inlineStr"/>
+      <c r="F285" t="inlineStr"/>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr"/>
+      <c r="E286" t="inlineStr"/>
+      <c r="F286" t="inlineStr"/>
+      <c r="G286" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-05
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G286"/>
+  <dimension ref="A1:G301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6652,9 +6652,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D272" t="inlineStr"/>
-      <c r="E272" t="inlineStr"/>
-      <c r="F272" t="inlineStr"/>
       <c r="G272" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6677,9 +6674,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D273" t="inlineStr"/>
-      <c r="E273" t="inlineStr"/>
-      <c r="F273" t="inlineStr"/>
       <c r="G273" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6702,9 +6696,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D274" t="inlineStr"/>
-      <c r="E274" t="inlineStr"/>
-      <c r="F274" t="inlineStr"/>
       <c r="G274" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6727,9 +6718,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D275" t="inlineStr"/>
-      <c r="E275" t="inlineStr"/>
-      <c r="F275" t="inlineStr"/>
       <c r="G275" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6752,9 +6740,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D276" t="inlineStr"/>
-      <c r="E276" t="inlineStr"/>
-      <c r="F276" t="inlineStr"/>
       <c r="G276" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6777,9 +6762,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D277" t="inlineStr"/>
-      <c r="E277" t="inlineStr"/>
-      <c r="F277" t="inlineStr"/>
       <c r="G277" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6802,9 +6784,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D278" t="inlineStr"/>
-      <c r="E278" t="inlineStr"/>
-      <c r="F278" t="inlineStr"/>
       <c r="G278" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6827,9 +6806,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D279" t="inlineStr"/>
-      <c r="E279" t="inlineStr"/>
-      <c r="F279" t="inlineStr"/>
       <c r="G279" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6852,9 +6828,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D280" t="inlineStr"/>
-      <c r="E280" t="inlineStr"/>
-      <c r="F280" t="inlineStr"/>
       <c r="G280" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6877,9 +6850,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D281" t="inlineStr"/>
-      <c r="E281" t="inlineStr"/>
-      <c r="F281" t="inlineStr"/>
       <c r="G281" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6902,9 +6872,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D282" t="inlineStr"/>
-      <c r="E282" t="inlineStr"/>
-      <c r="F282" t="inlineStr"/>
       <c r="G282" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6927,9 +6894,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D283" t="inlineStr"/>
-      <c r="E283" t="inlineStr"/>
-      <c r="F283" t="inlineStr"/>
       <c r="G283" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6952,9 +6916,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D284" t="inlineStr"/>
-      <c r="E284" t="inlineStr"/>
-      <c r="F284" t="inlineStr"/>
       <c r="G284" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -6977,9 +6938,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D285" t="inlineStr"/>
-      <c r="E285" t="inlineStr"/>
-      <c r="F285" t="inlineStr"/>
       <c r="G285" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7002,10 +6960,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D286" t="inlineStr"/>
-      <c r="E286" t="inlineStr"/>
-      <c r="F286" t="inlineStr"/>
       <c r="G286" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr"/>
+      <c r="E287" t="inlineStr"/>
+      <c r="F287" t="inlineStr"/>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr"/>
+      <c r="E288" t="inlineStr"/>
+      <c r="F288" t="inlineStr"/>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr"/>
+      <c r="E289" t="inlineStr"/>
+      <c r="F289" t="inlineStr"/>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr"/>
+      <c r="E290" t="inlineStr"/>
+      <c r="F290" t="inlineStr"/>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr"/>
+      <c r="E291" t="inlineStr"/>
+      <c r="F291" t="inlineStr"/>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr"/>
+      <c r="E292" t="inlineStr"/>
+      <c r="F292" t="inlineStr"/>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr"/>
+      <c r="E293" t="inlineStr"/>
+      <c r="F293" t="inlineStr"/>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr"/>
+      <c r="E294" t="inlineStr"/>
+      <c r="F294" t="inlineStr"/>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr"/>
+      <c r="E295" t="inlineStr"/>
+      <c r="F295" t="inlineStr"/>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr"/>
+      <c r="E296" t="inlineStr"/>
+      <c r="F296" t="inlineStr"/>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr"/>
+      <c r="E297" t="inlineStr"/>
+      <c r="F297" t="inlineStr"/>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr"/>
+      <c r="E298" t="inlineStr"/>
+      <c r="F298" t="inlineStr"/>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr"/>
+      <c r="E299" t="inlineStr"/>
+      <c r="F299" t="inlineStr"/>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr"/>
+      <c r="E300" t="inlineStr"/>
+      <c r="F300" t="inlineStr"/>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr"/>
+      <c r="E301" t="inlineStr"/>
+      <c r="F301" t="inlineStr"/>
+      <c r="G301" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-06
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G301"/>
+  <dimension ref="A1:G316"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6982,9 +6982,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D287" t="inlineStr"/>
-      <c r="E287" t="inlineStr"/>
-      <c r="F287" t="inlineStr"/>
       <c r="G287" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7007,9 +7004,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D288" t="inlineStr"/>
-      <c r="E288" t="inlineStr"/>
-      <c r="F288" t="inlineStr"/>
       <c r="G288" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7032,9 +7026,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D289" t="inlineStr"/>
-      <c r="E289" t="inlineStr"/>
-      <c r="F289" t="inlineStr"/>
       <c r="G289" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7057,9 +7048,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D290" t="inlineStr"/>
-      <c r="E290" t="inlineStr"/>
-      <c r="F290" t="inlineStr"/>
       <c r="G290" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7082,9 +7070,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D291" t="inlineStr"/>
-      <c r="E291" t="inlineStr"/>
-      <c r="F291" t="inlineStr"/>
       <c r="G291" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7107,9 +7092,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D292" t="inlineStr"/>
-      <c r="E292" t="inlineStr"/>
-      <c r="F292" t="inlineStr"/>
       <c r="G292" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7132,9 +7114,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D293" t="inlineStr"/>
-      <c r="E293" t="inlineStr"/>
-      <c r="F293" t="inlineStr"/>
       <c r="G293" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7157,9 +7136,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D294" t="inlineStr"/>
-      <c r="E294" t="inlineStr"/>
-      <c r="F294" t="inlineStr"/>
       <c r="G294" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7182,9 +7158,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D295" t="inlineStr"/>
-      <c r="E295" t="inlineStr"/>
-      <c r="F295" t="inlineStr"/>
       <c r="G295" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7207,9 +7180,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D296" t="inlineStr"/>
-      <c r="E296" t="inlineStr"/>
-      <c r="F296" t="inlineStr"/>
       <c r="G296" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7232,9 +7202,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D297" t="inlineStr"/>
-      <c r="E297" t="inlineStr"/>
-      <c r="F297" t="inlineStr"/>
       <c r="G297" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7257,9 +7224,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D298" t="inlineStr"/>
-      <c r="E298" t="inlineStr"/>
-      <c r="F298" t="inlineStr"/>
       <c r="G298" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7282,9 +7246,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D299" t="inlineStr"/>
-      <c r="E299" t="inlineStr"/>
-      <c r="F299" t="inlineStr"/>
       <c r="G299" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7307,9 +7268,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D300" t="inlineStr"/>
-      <c r="E300" t="inlineStr"/>
-      <c r="F300" t="inlineStr"/>
       <c r="G300" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7332,10 +7290,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D301" t="inlineStr"/>
-      <c r="E301" t="inlineStr"/>
-      <c r="F301" t="inlineStr"/>
       <c r="G301" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr"/>
+      <c r="E302" t="inlineStr"/>
+      <c r="F302" t="inlineStr"/>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr"/>
+      <c r="E303" t="inlineStr"/>
+      <c r="F303" t="inlineStr"/>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr"/>
+      <c r="E304" t="inlineStr"/>
+      <c r="F304" t="inlineStr"/>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr"/>
+      <c r="E305" t="inlineStr"/>
+      <c r="F305" t="inlineStr"/>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr"/>
+      <c r="E306" t="inlineStr"/>
+      <c r="F306" t="inlineStr"/>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr"/>
+      <c r="E307" t="inlineStr"/>
+      <c r="F307" t="inlineStr"/>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr"/>
+      <c r="E308" t="inlineStr"/>
+      <c r="F308" t="inlineStr"/>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr"/>
+      <c r="E309" t="inlineStr"/>
+      <c r="F309" t="inlineStr"/>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr"/>
+      <c r="E310" t="inlineStr"/>
+      <c r="F310" t="inlineStr"/>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr"/>
+      <c r="E311" t="inlineStr"/>
+      <c r="F311" t="inlineStr"/>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr"/>
+      <c r="E312" t="inlineStr"/>
+      <c r="F312" t="inlineStr"/>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr"/>
+      <c r="E313" t="inlineStr"/>
+      <c r="F313" t="inlineStr"/>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr"/>
+      <c r="E314" t="inlineStr"/>
+      <c r="F314" t="inlineStr"/>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr"/>
+      <c r="E315" t="inlineStr"/>
+      <c r="F315" t="inlineStr"/>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr"/>
+      <c r="E316" t="inlineStr"/>
+      <c r="F316" t="inlineStr"/>
+      <c r="G316" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-07
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G316"/>
+  <dimension ref="A1:G331"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7312,9 +7312,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D302" t="inlineStr"/>
-      <c r="E302" t="inlineStr"/>
-      <c r="F302" t="inlineStr"/>
       <c r="G302" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7337,9 +7334,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D303" t="inlineStr"/>
-      <c r="E303" t="inlineStr"/>
-      <c r="F303" t="inlineStr"/>
       <c r="G303" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7362,9 +7356,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D304" t="inlineStr"/>
-      <c r="E304" t="inlineStr"/>
-      <c r="F304" t="inlineStr"/>
       <c r="G304" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7387,9 +7378,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D305" t="inlineStr"/>
-      <c r="E305" t="inlineStr"/>
-      <c r="F305" t="inlineStr"/>
       <c r="G305" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7412,9 +7400,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D306" t="inlineStr"/>
-      <c r="E306" t="inlineStr"/>
-      <c r="F306" t="inlineStr"/>
       <c r="G306" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7437,9 +7422,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D307" t="inlineStr"/>
-      <c r="E307" t="inlineStr"/>
-      <c r="F307" t="inlineStr"/>
       <c r="G307" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7462,9 +7444,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D308" t="inlineStr"/>
-      <c r="E308" t="inlineStr"/>
-      <c r="F308" t="inlineStr"/>
       <c r="G308" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7487,9 +7466,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D309" t="inlineStr"/>
-      <c r="E309" t="inlineStr"/>
-      <c r="F309" t="inlineStr"/>
       <c r="G309" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7512,9 +7488,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D310" t="inlineStr"/>
-      <c r="E310" t="inlineStr"/>
-      <c r="F310" t="inlineStr"/>
       <c r="G310" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7537,9 +7510,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D311" t="inlineStr"/>
-      <c r="E311" t="inlineStr"/>
-      <c r="F311" t="inlineStr"/>
       <c r="G311" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7562,9 +7532,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D312" t="inlineStr"/>
-      <c r="E312" t="inlineStr"/>
-      <c r="F312" t="inlineStr"/>
       <c r="G312" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7587,9 +7554,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D313" t="inlineStr"/>
-      <c r="E313" t="inlineStr"/>
-      <c r="F313" t="inlineStr"/>
       <c r="G313" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7612,9 +7576,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D314" t="inlineStr"/>
-      <c r="E314" t="inlineStr"/>
-      <c r="F314" t="inlineStr"/>
       <c r="G314" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7637,9 +7598,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D315" t="inlineStr"/>
-      <c r="E315" t="inlineStr"/>
-      <c r="F315" t="inlineStr"/>
       <c r="G315" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7662,10 +7620,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D316" t="inlineStr"/>
-      <c r="E316" t="inlineStr"/>
-      <c r="F316" t="inlineStr"/>
       <c r="G316" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr"/>
+      <c r="E317" t="inlineStr"/>
+      <c r="F317" t="inlineStr"/>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr"/>
+      <c r="E318" t="inlineStr"/>
+      <c r="F318" t="inlineStr"/>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr"/>
+      <c r="E319" t="inlineStr"/>
+      <c r="F319" t="inlineStr"/>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr"/>
+      <c r="E320" t="inlineStr"/>
+      <c r="F320" t="inlineStr"/>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr"/>
+      <c r="E321" t="inlineStr"/>
+      <c r="F321" t="inlineStr"/>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr"/>
+      <c r="E322" t="inlineStr"/>
+      <c r="F322" t="inlineStr"/>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr"/>
+      <c r="E323" t="inlineStr"/>
+      <c r="F323" t="inlineStr"/>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr"/>
+      <c r="E324" t="inlineStr"/>
+      <c r="F324" t="inlineStr"/>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr"/>
+      <c r="E325" t="inlineStr"/>
+      <c r="F325" t="inlineStr"/>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr"/>
+      <c r="E326" t="inlineStr"/>
+      <c r="F326" t="inlineStr"/>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr"/>
+      <c r="E327" t="inlineStr"/>
+      <c r="F327" t="inlineStr"/>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr"/>
+      <c r="E328" t="inlineStr"/>
+      <c r="F328" t="inlineStr"/>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr"/>
+      <c r="E329" t="inlineStr"/>
+      <c r="F329" t="inlineStr"/>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr"/>
+      <c r="E330" t="inlineStr"/>
+      <c r="F330" t="inlineStr"/>
+      <c r="G330" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr"/>
+      <c r="E331" t="inlineStr"/>
+      <c r="F331" t="inlineStr"/>
+      <c r="G331" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-08
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G331"/>
+  <dimension ref="A1:G346"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7642,9 +7642,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D317" t="inlineStr"/>
-      <c r="E317" t="inlineStr"/>
-      <c r="F317" t="inlineStr"/>
       <c r="G317" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7667,9 +7664,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D318" t="inlineStr"/>
-      <c r="E318" t="inlineStr"/>
-      <c r="F318" t="inlineStr"/>
       <c r="G318" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7692,9 +7686,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D319" t="inlineStr"/>
-      <c r="E319" t="inlineStr"/>
-      <c r="F319" t="inlineStr"/>
       <c r="G319" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7717,9 +7708,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D320" t="inlineStr"/>
-      <c r="E320" t="inlineStr"/>
-      <c r="F320" t="inlineStr"/>
       <c r="G320" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7742,9 +7730,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D321" t="inlineStr"/>
-      <c r="E321" t="inlineStr"/>
-      <c r="F321" t="inlineStr"/>
       <c r="G321" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7767,9 +7752,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D322" t="inlineStr"/>
-      <c r="E322" t="inlineStr"/>
-      <c r="F322" t="inlineStr"/>
       <c r="G322" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7792,9 +7774,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D323" t="inlineStr"/>
-      <c r="E323" t="inlineStr"/>
-      <c r="F323" t="inlineStr"/>
       <c r="G323" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7817,9 +7796,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D324" t="inlineStr"/>
-      <c r="E324" t="inlineStr"/>
-      <c r="F324" t="inlineStr"/>
       <c r="G324" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7842,9 +7818,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D325" t="inlineStr"/>
-      <c r="E325" t="inlineStr"/>
-      <c r="F325" t="inlineStr"/>
       <c r="G325" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7867,9 +7840,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D326" t="inlineStr"/>
-      <c r="E326" t="inlineStr"/>
-      <c r="F326" t="inlineStr"/>
       <c r="G326" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7892,9 +7862,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D327" t="inlineStr"/>
-      <c r="E327" t="inlineStr"/>
-      <c r="F327" t="inlineStr"/>
       <c r="G327" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7917,9 +7884,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D328" t="inlineStr"/>
-      <c r="E328" t="inlineStr"/>
-      <c r="F328" t="inlineStr"/>
       <c r="G328" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7942,9 +7906,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D329" t="inlineStr"/>
-      <c r="E329" t="inlineStr"/>
-      <c r="F329" t="inlineStr"/>
       <c r="G329" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7967,9 +7928,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D330" t="inlineStr"/>
-      <c r="E330" t="inlineStr"/>
-      <c r="F330" t="inlineStr"/>
       <c r="G330" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7992,10 +7950,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D331" t="inlineStr"/>
-      <c r="E331" t="inlineStr"/>
-      <c r="F331" t="inlineStr"/>
       <c r="G331" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr"/>
+      <c r="E332" t="inlineStr"/>
+      <c r="F332" t="inlineStr"/>
+      <c r="G332" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr"/>
+      <c r="E333" t="inlineStr"/>
+      <c r="F333" t="inlineStr"/>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr"/>
+      <c r="E334" t="inlineStr"/>
+      <c r="F334" t="inlineStr"/>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr"/>
+      <c r="E335" t="inlineStr"/>
+      <c r="F335" t="inlineStr"/>
+      <c r="G335" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr"/>
+      <c r="E336" t="inlineStr"/>
+      <c r="F336" t="inlineStr"/>
+      <c r="G336" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr"/>
+      <c r="E337" t="inlineStr"/>
+      <c r="F337" t="inlineStr"/>
+      <c r="G337" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr"/>
+      <c r="E338" t="inlineStr"/>
+      <c r="F338" t="inlineStr"/>
+      <c r="G338" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr"/>
+      <c r="E339" t="inlineStr"/>
+      <c r="F339" t="inlineStr"/>
+      <c r="G339" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr"/>
+      <c r="E340" t="inlineStr"/>
+      <c r="F340" t="inlineStr"/>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr"/>
+      <c r="E341" t="inlineStr"/>
+      <c r="F341" t="inlineStr"/>
+      <c r="G341" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr"/>
+      <c r="E342" t="inlineStr"/>
+      <c r="F342" t="inlineStr"/>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr"/>
+      <c r="E343" t="inlineStr"/>
+      <c r="F343" t="inlineStr"/>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr"/>
+      <c r="E344" t="inlineStr"/>
+      <c r="F344" t="inlineStr"/>
+      <c r="G344" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr"/>
+      <c r="E345" t="inlineStr"/>
+      <c r="F345" t="inlineStr"/>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr"/>
+      <c r="E346" t="inlineStr"/>
+      <c r="F346" t="inlineStr"/>
+      <c r="G346" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-09
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G346"/>
+  <dimension ref="A1:G361"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7972,9 +7972,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D332" t="inlineStr"/>
-      <c r="E332" t="inlineStr"/>
-      <c r="F332" t="inlineStr"/>
       <c r="G332" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -7997,9 +7994,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D333" t="inlineStr"/>
-      <c r="E333" t="inlineStr"/>
-      <c r="F333" t="inlineStr"/>
       <c r="G333" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8022,9 +8016,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D334" t="inlineStr"/>
-      <c r="E334" t="inlineStr"/>
-      <c r="F334" t="inlineStr"/>
       <c r="G334" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8047,9 +8038,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D335" t="inlineStr"/>
-      <c r="E335" t="inlineStr"/>
-      <c r="F335" t="inlineStr"/>
       <c r="G335" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8072,9 +8060,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D336" t="inlineStr"/>
-      <c r="E336" t="inlineStr"/>
-      <c r="F336" t="inlineStr"/>
       <c r="G336" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8097,9 +8082,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D337" t="inlineStr"/>
-      <c r="E337" t="inlineStr"/>
-      <c r="F337" t="inlineStr"/>
       <c r="G337" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8122,9 +8104,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D338" t="inlineStr"/>
-      <c r="E338" t="inlineStr"/>
-      <c r="F338" t="inlineStr"/>
       <c r="G338" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8147,9 +8126,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D339" t="inlineStr"/>
-      <c r="E339" t="inlineStr"/>
-      <c r="F339" t="inlineStr"/>
       <c r="G339" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8172,9 +8148,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D340" t="inlineStr"/>
-      <c r="E340" t="inlineStr"/>
-      <c r="F340" t="inlineStr"/>
       <c r="G340" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8197,9 +8170,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D341" t="inlineStr"/>
-      <c r="E341" t="inlineStr"/>
-      <c r="F341" t="inlineStr"/>
       <c r="G341" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8222,9 +8192,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D342" t="inlineStr"/>
-      <c r="E342" t="inlineStr"/>
-      <c r="F342" t="inlineStr"/>
       <c r="G342" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8247,9 +8214,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D343" t="inlineStr"/>
-      <c r="E343" t="inlineStr"/>
-      <c r="F343" t="inlineStr"/>
       <c r="G343" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8272,9 +8236,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D344" t="inlineStr"/>
-      <c r="E344" t="inlineStr"/>
-      <c r="F344" t="inlineStr"/>
       <c r="G344" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8297,9 +8258,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D345" t="inlineStr"/>
-      <c r="E345" t="inlineStr"/>
-      <c r="F345" t="inlineStr"/>
       <c r="G345" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8322,10 +8280,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D346" t="inlineStr"/>
-      <c r="E346" t="inlineStr"/>
-      <c r="F346" t="inlineStr"/>
       <c r="G346" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr"/>
+      <c r="E347" t="inlineStr"/>
+      <c r="F347" t="inlineStr"/>
+      <c r="G347" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr"/>
+      <c r="E348" t="inlineStr"/>
+      <c r="F348" t="inlineStr"/>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr"/>
+      <c r="E349" t="inlineStr"/>
+      <c r="F349" t="inlineStr"/>
+      <c r="G349" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr"/>
+      <c r="E350" t="inlineStr"/>
+      <c r="F350" t="inlineStr"/>
+      <c r="G350" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr"/>
+      <c r="E351" t="inlineStr"/>
+      <c r="F351" t="inlineStr"/>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr"/>
+      <c r="E352" t="inlineStr"/>
+      <c r="F352" t="inlineStr"/>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr"/>
+      <c r="E353" t="inlineStr"/>
+      <c r="F353" t="inlineStr"/>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr"/>
+      <c r="E354" t="inlineStr"/>
+      <c r="F354" t="inlineStr"/>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr"/>
+      <c r="E355" t="inlineStr"/>
+      <c r="F355" t="inlineStr"/>
+      <c r="G355" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr"/>
+      <c r="E356" t="inlineStr"/>
+      <c r="F356" t="inlineStr"/>
+      <c r="G356" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr"/>
+      <c r="E357" t="inlineStr"/>
+      <c r="F357" t="inlineStr"/>
+      <c r="G357" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr"/>
+      <c r="E358" t="inlineStr"/>
+      <c r="F358" t="inlineStr"/>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr"/>
+      <c r="E359" t="inlineStr"/>
+      <c r="F359" t="inlineStr"/>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr"/>
+      <c r="E360" t="inlineStr"/>
+      <c r="F360" t="inlineStr"/>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr"/>
+      <c r="E361" t="inlineStr"/>
+      <c r="F361" t="inlineStr"/>
+      <c r="G361" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-10
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G361"/>
+  <dimension ref="A1:G376"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8302,9 +8302,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D347" t="inlineStr"/>
-      <c r="E347" t="inlineStr"/>
-      <c r="F347" t="inlineStr"/>
       <c r="G347" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8327,9 +8324,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D348" t="inlineStr"/>
-      <c r="E348" t="inlineStr"/>
-      <c r="F348" t="inlineStr"/>
       <c r="G348" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8352,9 +8346,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D349" t="inlineStr"/>
-      <c r="E349" t="inlineStr"/>
-      <c r="F349" t="inlineStr"/>
       <c r="G349" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8377,9 +8368,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D350" t="inlineStr"/>
-      <c r="E350" t="inlineStr"/>
-      <c r="F350" t="inlineStr"/>
       <c r="G350" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8402,9 +8390,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D351" t="inlineStr"/>
-      <c r="E351" t="inlineStr"/>
-      <c r="F351" t="inlineStr"/>
       <c r="G351" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8427,9 +8412,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D352" t="inlineStr"/>
-      <c r="E352" t="inlineStr"/>
-      <c r="F352" t="inlineStr"/>
       <c r="G352" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8452,9 +8434,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D353" t="inlineStr"/>
-      <c r="E353" t="inlineStr"/>
-      <c r="F353" t="inlineStr"/>
       <c r="G353" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8477,9 +8456,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D354" t="inlineStr"/>
-      <c r="E354" t="inlineStr"/>
-      <c r="F354" t="inlineStr"/>
       <c r="G354" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8502,9 +8478,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D355" t="inlineStr"/>
-      <c r="E355" t="inlineStr"/>
-      <c r="F355" t="inlineStr"/>
       <c r="G355" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8527,9 +8500,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D356" t="inlineStr"/>
-      <c r="E356" t="inlineStr"/>
-      <c r="F356" t="inlineStr"/>
       <c r="G356" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8552,9 +8522,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D357" t="inlineStr"/>
-      <c r="E357" t="inlineStr"/>
-      <c r="F357" t="inlineStr"/>
       <c r="G357" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8577,9 +8544,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D358" t="inlineStr"/>
-      <c r="E358" t="inlineStr"/>
-      <c r="F358" t="inlineStr"/>
       <c r="G358" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8602,9 +8566,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D359" t="inlineStr"/>
-      <c r="E359" t="inlineStr"/>
-      <c r="F359" t="inlineStr"/>
       <c r="G359" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8627,9 +8588,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D360" t="inlineStr"/>
-      <c r="E360" t="inlineStr"/>
-      <c r="F360" t="inlineStr"/>
       <c r="G360" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8652,10 +8610,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D361" t="inlineStr"/>
-      <c r="E361" t="inlineStr"/>
-      <c r="F361" t="inlineStr"/>
       <c r="G361" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr"/>
+      <c r="E362" t="inlineStr"/>
+      <c r="F362" t="inlineStr"/>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr"/>
+      <c r="E363" t="inlineStr"/>
+      <c r="F363" t="inlineStr"/>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr"/>
+      <c r="E364" t="inlineStr"/>
+      <c r="F364" t="inlineStr"/>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr"/>
+      <c r="E365" t="inlineStr"/>
+      <c r="F365" t="inlineStr"/>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr"/>
+      <c r="E366" t="inlineStr"/>
+      <c r="F366" t="inlineStr"/>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr"/>
+      <c r="E367" t="inlineStr"/>
+      <c r="F367" t="inlineStr"/>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr"/>
+      <c r="E368" t="inlineStr"/>
+      <c r="F368" t="inlineStr"/>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr"/>
+      <c r="E369" t="inlineStr"/>
+      <c r="F369" t="inlineStr"/>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr"/>
+      <c r="E370" t="inlineStr"/>
+      <c r="F370" t="inlineStr"/>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr"/>
+      <c r="E371" t="inlineStr"/>
+      <c r="F371" t="inlineStr"/>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr"/>
+      <c r="E372" t="inlineStr"/>
+      <c r="F372" t="inlineStr"/>
+      <c r="G372" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr"/>
+      <c r="E373" t="inlineStr"/>
+      <c r="F373" t="inlineStr"/>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr"/>
+      <c r="E374" t="inlineStr"/>
+      <c r="F374" t="inlineStr"/>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr"/>
+      <c r="E375" t="inlineStr"/>
+      <c r="F375" t="inlineStr"/>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr"/>
+      <c r="E376" t="inlineStr"/>
+      <c r="F376" t="inlineStr"/>
+      <c r="G376" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-11
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G376"/>
+  <dimension ref="A1:G391"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8632,9 +8632,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D362" t="inlineStr"/>
-      <c r="E362" t="inlineStr"/>
-      <c r="F362" t="inlineStr"/>
       <c r="G362" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8657,9 +8654,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D363" t="inlineStr"/>
-      <c r="E363" t="inlineStr"/>
-      <c r="F363" t="inlineStr"/>
       <c r="G363" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8682,9 +8676,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D364" t="inlineStr"/>
-      <c r="E364" t="inlineStr"/>
-      <c r="F364" t="inlineStr"/>
       <c r="G364" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8707,9 +8698,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D365" t="inlineStr"/>
-      <c r="E365" t="inlineStr"/>
-      <c r="F365" t="inlineStr"/>
       <c r="G365" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8732,9 +8720,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D366" t="inlineStr"/>
-      <c r="E366" t="inlineStr"/>
-      <c r="F366" t="inlineStr"/>
       <c r="G366" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8757,9 +8742,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D367" t="inlineStr"/>
-      <c r="E367" t="inlineStr"/>
-      <c r="F367" t="inlineStr"/>
       <c r="G367" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8782,9 +8764,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D368" t="inlineStr"/>
-      <c r="E368" t="inlineStr"/>
-      <c r="F368" t="inlineStr"/>
       <c r="G368" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8807,9 +8786,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D369" t="inlineStr"/>
-      <c r="E369" t="inlineStr"/>
-      <c r="F369" t="inlineStr"/>
       <c r="G369" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8832,9 +8808,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D370" t="inlineStr"/>
-      <c r="E370" t="inlineStr"/>
-      <c r="F370" t="inlineStr"/>
       <c r="G370" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8857,9 +8830,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D371" t="inlineStr"/>
-      <c r="E371" t="inlineStr"/>
-      <c r="F371" t="inlineStr"/>
       <c r="G371" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8882,9 +8852,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D372" t="inlineStr"/>
-      <c r="E372" t="inlineStr"/>
-      <c r="F372" t="inlineStr"/>
       <c r="G372" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8907,9 +8874,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D373" t="inlineStr"/>
-      <c r="E373" t="inlineStr"/>
-      <c r="F373" t="inlineStr"/>
       <c r="G373" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8932,9 +8896,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D374" t="inlineStr"/>
-      <c r="E374" t="inlineStr"/>
-      <c r="F374" t="inlineStr"/>
       <c r="G374" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8957,9 +8918,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D375" t="inlineStr"/>
-      <c r="E375" t="inlineStr"/>
-      <c r="F375" t="inlineStr"/>
       <c r="G375" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -8982,10 +8940,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D376" t="inlineStr"/>
-      <c r="E376" t="inlineStr"/>
-      <c r="F376" t="inlineStr"/>
       <c r="G376" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr"/>
+      <c r="E377" t="inlineStr"/>
+      <c r="F377" t="inlineStr"/>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='api.scraperapi.com', port=443): Read timed out. (read timeout=60)</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr"/>
+      <c r="E378" t="inlineStr"/>
+      <c r="F378" t="inlineStr"/>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>HTTPSConnectionPool(host='api.scraperapi.com', port=443): Read timed out. (read timeout=60)</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr"/>
+      <c r="E379" t="inlineStr"/>
+      <c r="F379" t="inlineStr"/>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr"/>
+      <c r="E380" t="inlineStr"/>
+      <c r="F380" t="inlineStr"/>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr"/>
+      <c r="E381" t="inlineStr"/>
+      <c r="F381" t="inlineStr"/>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr"/>
+      <c r="E382" t="inlineStr"/>
+      <c r="F382" t="inlineStr"/>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr"/>
+      <c r="E383" t="inlineStr"/>
+      <c r="F383" t="inlineStr"/>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr"/>
+      <c r="E384" t="inlineStr"/>
+      <c r="F384" t="inlineStr"/>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr"/>
+      <c r="E385" t="inlineStr"/>
+      <c r="F385" t="inlineStr"/>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr"/>
+      <c r="E386" t="inlineStr"/>
+      <c r="F386" t="inlineStr"/>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr"/>
+      <c r="E387" t="inlineStr"/>
+      <c r="F387" t="inlineStr"/>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr"/>
+      <c r="E388" t="inlineStr"/>
+      <c r="F388" t="inlineStr"/>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr"/>
+      <c r="E389" t="inlineStr"/>
+      <c r="F389" t="inlineStr"/>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr"/>
+      <c r="E390" t="inlineStr"/>
+      <c r="F390" t="inlineStr"/>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr"/>
+      <c r="E391" t="inlineStr"/>
+      <c r="F391" t="inlineStr"/>
+      <c r="G391" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>

<commit_message>
Atualiza preços de 2026-09-12
</commit_message>
<xml_diff>
--- a/precos-eletrodomesticos/data/historico.xlsx
+++ b/precos-eletrodomesticos/data/historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G391"/>
+  <dimension ref="A1:G406"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8962,9 +8962,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D377" t="inlineStr"/>
-      <c r="E377" t="inlineStr"/>
-      <c r="F377" t="inlineStr"/>
       <c r="G377" t="inlineStr">
         <is>
           <t>HTTPSConnectionPool(host='api.scraperapi.com', port=443): Read timed out. (read timeout=60)</t>
@@ -8987,9 +8984,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D378" t="inlineStr"/>
-      <c r="E378" t="inlineStr"/>
-      <c r="F378" t="inlineStr"/>
       <c r="G378" t="inlineStr">
         <is>
           <t>HTTPSConnectionPool(host='api.scraperapi.com', port=443): Read timed out. (read timeout=60)</t>
@@ -9012,9 +9006,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D379" t="inlineStr"/>
-      <c r="E379" t="inlineStr"/>
-      <c r="F379" t="inlineStr"/>
       <c r="G379" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9037,9 +9028,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D380" t="inlineStr"/>
-      <c r="E380" t="inlineStr"/>
-      <c r="F380" t="inlineStr"/>
       <c r="G380" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9062,9 +9050,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D381" t="inlineStr"/>
-      <c r="E381" t="inlineStr"/>
-      <c r="F381" t="inlineStr"/>
       <c r="G381" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9087,9 +9072,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D382" t="inlineStr"/>
-      <c r="E382" t="inlineStr"/>
-      <c r="F382" t="inlineStr"/>
       <c r="G382" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9112,9 +9094,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D383" t="inlineStr"/>
-      <c r="E383" t="inlineStr"/>
-      <c r="F383" t="inlineStr"/>
       <c r="G383" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9137,9 +9116,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D384" t="inlineStr"/>
-      <c r="E384" t="inlineStr"/>
-      <c r="F384" t="inlineStr"/>
       <c r="G384" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9162,9 +9138,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D385" t="inlineStr"/>
-      <c r="E385" t="inlineStr"/>
-      <c r="F385" t="inlineStr"/>
       <c r="G385" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9187,9 +9160,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D386" t="inlineStr"/>
-      <c r="E386" t="inlineStr"/>
-      <c r="F386" t="inlineStr"/>
       <c r="G386" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9212,9 +9182,6 @@
           <t>Mercado Livre</t>
         </is>
       </c>
-      <c r="D387" t="inlineStr"/>
-      <c r="E387" t="inlineStr"/>
-      <c r="F387" t="inlineStr"/>
       <c r="G387" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9237,9 +9204,6 @@
           <t>Casas Bahia</t>
         </is>
       </c>
-      <c r="D388" t="inlineStr"/>
-      <c r="E388" t="inlineStr"/>
-      <c r="F388" t="inlineStr"/>
       <c r="G388" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9262,9 +9226,6 @@
           <t>Fast Shop</t>
         </is>
       </c>
-      <c r="D389" t="inlineStr"/>
-      <c r="E389" t="inlineStr"/>
-      <c r="F389" t="inlineStr"/>
       <c r="G389" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9287,9 +9248,6 @@
           <t>Magazine Luiza</t>
         </is>
       </c>
-      <c r="D390" t="inlineStr"/>
-      <c r="E390" t="inlineStr"/>
-      <c r="F390" t="inlineStr"/>
       <c r="G390" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
@@ -9312,10 +9270,382 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D391" t="inlineStr"/>
-      <c r="E391" t="inlineStr"/>
-      <c r="F391" t="inlineStr"/>
       <c r="G391" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr"/>
+      <c r="E392" t="inlineStr"/>
+      <c r="F392" t="inlineStr"/>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr"/>
+      <c r="E393" t="inlineStr"/>
+      <c r="F393" t="inlineStr"/>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr"/>
+      <c r="E394" t="inlineStr"/>
+      <c r="F394" t="inlineStr"/>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr"/>
+      <c r="E395" t="inlineStr"/>
+      <c r="F395" t="inlineStr"/>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>Geladeira Brastemp Frost Free 375L</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr"/>
+      <c r="E396" t="inlineStr"/>
+      <c r="F396" t="inlineStr"/>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr"/>
+      <c r="E397" t="inlineStr"/>
+      <c r="F397" t="inlineStr"/>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr"/>
+      <c r="E398" t="inlineStr"/>
+      <c r="F398" t="inlineStr"/>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr"/>
+      <c r="E399" t="inlineStr"/>
+      <c r="F399" t="inlineStr"/>
+      <c r="G399" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr"/>
+      <c r="E400" t="inlineStr"/>
+      <c r="F400" t="inlineStr"/>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>Micro-ondas Electrolux 20L</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr"/>
+      <c r="E401" t="inlineStr"/>
+      <c r="F401" t="inlineStr"/>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr"/>
+      <c r="E402" t="inlineStr"/>
+      <c r="F402" t="inlineStr"/>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>Casas Bahia</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr"/>
+      <c r="E403" t="inlineStr"/>
+      <c r="F403" t="inlineStr"/>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Fast Shop</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr"/>
+      <c r="E404" t="inlineStr"/>
+      <c r="F404" t="inlineStr"/>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Magazine Luiza</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr"/>
+      <c r="E405" t="inlineStr"/>
+      <c r="F405" t="inlineStr"/>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>Fogão 4 bocas Consul</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr"/>
+      <c r="E406" t="inlineStr"/>
+      <c r="F406" t="inlineStr"/>
+      <c r="G406" t="inlineStr">
         <is>
           <t>403 do proxy: 'You have exhausted the API Credits available in this monthly cycle. You can upgrade your subscription or enable overages from your dashboard (https://dashboard.scraperapi.com/billing). For custom plan upgrades, please contact support (https://www.scraperapi.com/support/).'</t>
         </is>

</xml_diff>